<commit_message>
ready app with lists of branches
</commit_message>
<xml_diff>
--- a/scripts/e2e-tmp/import.xlsx
+++ b/scripts/e2e-tmp/import.xlsx
@@ -442,16 +442,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>استيراد1 09897998</v>
+        <v>استيراد1 76676885</v>
       </c>
       <c r="B2" t="str">
-        <v>078098979981</v>
+        <v>078766768851</v>
       </c>
       <c r="C2" t="str">
         <v>1234567890</v>
       </c>
       <c r="D2" t="str">
-        <v>IMP109897998</v>
+        <v>IMP176676885</v>
       </c>
       <c r="E2" t="str">
         <v>شيك</v>
@@ -483,16 +483,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>استيراد2 09897998</v>
+        <v>استيراد2 76676885</v>
       </c>
       <c r="B3" t="str">
-        <v>078098979982</v>
+        <v>078766768852</v>
       </c>
       <c r="C3" t="str">
         <v>1234567891</v>
       </c>
       <c r="D3" t="str">
-        <v>IMP209897998</v>
+        <v>IMP276676885</v>
       </c>
       <c r="E3" t="str">
         <v>شيك</v>

</xml_diff>